<commit_message>
update for report send to email feature
</commit_message>
<xml_diff>
--- a/data/DataUser.xlsx
+++ b/data/DataUser.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CodeProject\Java\MyProject\CucumberBDDProject\CucumberMiniFramework\cucumber_hybrid_framework\data\"/>
     </mc:Choice>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>EMAIL</t>
   </si>
@@ -37,12 +37,25 @@
   </si>
   <si>
     <t>Mo0^f1ZG</t>
+  </si>
+  <si>
+    <t>claud.kohler@gmail.com</t>
+  </si>
+  <si>
+    <t>Ys6^PCdF</t>
+  </si>
+  <si>
+    <t>alline.mayer@hotmail.com</t>
+  </si>
+  <si>
+    <t>Yy0*P1t%</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -408,27 +421,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{290CBC4D-1AFC-4B6D-8F9B-23F8520A0F28}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="28.140625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="10.85546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>